<commit_message>
Add verification for scenario where all node responses are error, and rename test cases
</commit_message>
<xml_diff>
--- a/InputFiles/API/Federation/AllowedValues.xlsx
+++ b/InputFiles/API/Federation/AllowedValues.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leungvw/git2/Commons_Automation/InputFiles/API/Federation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88207591-BE1A-B746-B2CB-B08F6F3DFB4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1765567C-A3D7-AE4B-9E0D-2CCB151281ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19140" yWindow="-25920" windowWidth="28040" windowHeight="17440" firstSheet="1" activeTab="13" xr2:uid="{8F72063A-9150-2546-A2F6-5AE255D363FD}"/>
+    <workbookView xWindow="13180" yWindow="2780" windowWidth="33760" windowHeight="22160" firstSheet="1" activeTab="14" xr2:uid="{8F72063A-9150-2546-A2F6-5AE255D363FD}"/>
   </bookViews>
   <sheets>
     <sheet name="FileType" sheetId="2" r:id="rId1"/>
@@ -27,6 +27,7 @@
     <sheet name="SampTiss" sheetId="13" r:id="rId12"/>
     <sheet name="SampTumor" sheetId="14" r:id="rId13"/>
     <sheet name="SampTumGrd" sheetId="15" r:id="rId14"/>
+    <sheet name="SampDiagCat" sheetId="16" r:id="rId15"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="214">
   <si>
     <t>ADF</t>
   </si>
@@ -598,6 +599,99 @@
   </si>
   <si>
     <t>Not Applicable</t>
+  </si>
+  <si>
+    <t>Atypical Teratoid/Rhabdoid Tumors</t>
+  </si>
+  <si>
+    <t>Choroid Plexus Tumors</t>
+  </si>
+  <si>
+    <t>CNS Germ Cell Tumors</t>
+  </si>
+  <si>
+    <t>CNS Sarcomas</t>
+  </si>
+  <si>
+    <t>Craniopharyngiomas</t>
+  </si>
+  <si>
+    <t>Endocrine and Neuroendocrine Tumors</t>
+  </si>
+  <si>
+    <t>Ependymoma</t>
+  </si>
+  <si>
+    <t>Ewings Sarcoma</t>
+  </si>
+  <si>
+    <t>Germ Cell Tumors</t>
+  </si>
+  <si>
+    <t>Glioneuronal and Neuronal Tumors</t>
+  </si>
+  <si>
+    <t>High-Grade Glioma</t>
+  </si>
+  <si>
+    <t>Hodgkin Lymphoma</t>
+  </si>
+  <si>
+    <t>Liver Tumors</t>
+  </si>
+  <si>
+    <t>Low-Grade Gliomas</t>
+  </si>
+  <si>
+    <t>Lymphoblastic Leukemia</t>
+  </si>
+  <si>
+    <t>Lymphoproliferative Diseases</t>
+  </si>
+  <si>
+    <t>Medulloblastoma</t>
+  </si>
+  <si>
+    <t>Myeloid Leukemia</t>
+  </si>
+  <si>
+    <t>Neuroblastoma</t>
+  </si>
+  <si>
+    <t>Non-Hodgkin Lymphoma</t>
+  </si>
+  <si>
+    <t>Osteosarcoma</t>
+  </si>
+  <si>
+    <t>Other Brain Tumors</t>
+  </si>
+  <si>
+    <t>Other CNS Embryonal Tumors</t>
+  </si>
+  <si>
+    <t>Other Gliomas</t>
+  </si>
+  <si>
+    <t>Other Hematopoietic Tumors</t>
+  </si>
+  <si>
+    <t>Other Solid Tumors</t>
+  </si>
+  <si>
+    <t>Renal Tumors</t>
+  </si>
+  <si>
+    <t>Retinoblastoma</t>
+  </si>
+  <si>
+    <t>Rhabdoid Tumors</t>
+  </si>
+  <si>
+    <t>Rhabdomyosarcoma</t>
+  </si>
+  <si>
+    <t>Soft Tissue Tumors</t>
   </si>
 </sst>
 </file>
@@ -1632,6 +1726,174 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88C0E17D-CBFA-954E-A3BD-DD9F2EB1B3C9}">
+  <dimension ref="A1:A31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="33" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>213</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C1D6B96-7285-604A-81E3-2DB1C7B968A4}">
   <dimension ref="A1:A5"/>

</xml_diff>